<commit_message>
fix(statements): match native MT4 DetailedStatement HTML format, stats, and balance graph
</commit_message>
<xml_diff>
--- a/docs/Hedge_Optimization_Calculator.xlsx
+++ b/docs/Hedge_Optimization_Calculator.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\Documents\dev\TradeDashboard\TradeDashboardPY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\Documents\dev\TradeDashboard\TradeDashboardPY\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1979BB8-B8B9-4155-BD12-1E2D37636FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1999C4A-315B-499B-A8B0-33C86A98CA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="1140" windowWidth="16040" windowHeight="8220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="9270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hedge Optimization" sheetId="1" r:id="rId1"/>
@@ -508,7 +508,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>50000</v>
+        <v>2183000</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -516,7 +516,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>25</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -533,7 +533,7 @@
       </c>
       <c r="B5" s="2">
         <f>B3*B4</f>
-        <v>2500000</v>
+        <v>50000000</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -547,7 +547,7 @@
         <v>5</v>
       </c>
       <c r="B8">
-        <v>100</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -564,7 +564,7 @@
       </c>
       <c r="B10" s="2">
         <f>B5*(B9/B8)</f>
-        <v>12500</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -578,7 +578,7 @@
         <v>5</v>
       </c>
       <c r="B13">
-        <v>400</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -595,7 +595,7 @@
       </c>
       <c r="B15" s="2">
         <f>B5*(B14/B13)</f>
-        <v>5000</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -610,7 +610,7 @@
       </c>
       <c r="B18" s="2">
         <f>(B2/2)+((B10-B15)/2)</f>
-        <v>28750</v>
+        <v>904000</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -619,7 +619,7 @@
       </c>
       <c r="B19" s="2">
         <f>(B2/2)-((B10-B15)/2)</f>
-        <v>21250</v>
+        <v>1279000</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -634,7 +634,7 @@
       </c>
       <c r="B22" s="4">
         <f>B18/B2</f>
-        <v>0.57499999999999996</v>
+        <v>0.41410902427851581</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -643,7 +643,7 @@
       </c>
       <c r="B23" s="4">
         <f>B19/B2</f>
-        <v>0.42499999999999999</v>
+        <v>0.58589097572148419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>